<commit_message>
Add 8 blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (17):
- blocks/accordion-faq/accordion-faq.css
- blocks/cards-business/cards-business.css
- blocks/cards-future/cards-future.css
- blocks/cards-news/cards-news.css
- blocks/cards-performance/cards-performance.css
- blocks/cards-purpose/cards-purpose.css
- blocks/cards-work/cards-work.css
- blocks/carousel-hero/carousel-hero.css
- head.html
- styles/fonts.css
- styles/styles.css
- tools/importer/import-homepage.bundle.js
- tools/importer/import-homepage.js
- tools/importer/page-templates.json
- tools/importer/parsers/accordion-faq.js
- tools/importer/reports/import-homepage.report.xlsx
- tools/importer/reports/index.report.json
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -40,7 +40,7 @@
     <t>index.report.json</t>
   </si>
   <si>
-    <t>["carousel-hero","cards-business","cards-purpose","cards-performance","cards-performance","cards-future","cards-news","cards-work","accordion-faq"]</t>
+    <t>["carousel-hero","cards-business","cards-purpose","cards-performance","cards-future","cards-news","cards-work","accordion-faq"]</t>
   </si>
   <si>
     <t>index</t>
@@ -52,7 +52,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-04-21T08:24:23.579Z</t>
+    <t>2026-04-21T09:33:21.904Z</t>
   </si>
   <si>
     <t>The Mahindra Group Official Website | Together We Rise</t>

</xml_diff>